<commit_message>
[feat/ASP-7977-Device-Name-Redesign] TB Workload and device activity fixed formatting
</commit_message>
<xml_diff>
--- a/api/templates/device_activity/uk.xlsx
+++ b/api/templates/device_activity/uk.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{579484CA-675A-5143-90D2-92ECE91D8233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Підсумки діяльності" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Деталізація по пробам" state="visible" r:id="rId5"/>
+    <sheet name="Підсумки діяльності" sheetId="1" r:id="rId1"/>
+    <sheet name="Деталізація по пробам" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -50,7 +51,7 @@
     <t>Оновлення останнього результату</t>
   </si>
   <si>
-    <t xml:space="preserve">Статус технічного
+    <t>Статус технічного
 обслуговування</t>
   </si>
   <si>
@@ -93,39 +94,40 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="[$-409]mmmm d&quot;, &quot;yyyy;@"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
-      <color rgb="FF000000"/>
-      <family val="2"/>
-      <sz val="16"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
-      <color rgb="FF000000"/>
-      <family val="2"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <charset val="1"/>
-      <family val="2"/>
       <sz val="12"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -142,7 +144,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -151,27 +153,65 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium"/>
-      <right style="medium"/>
-      <top style="medium"/>
-      <bottom style="medium"/>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="slantDashDot">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,150 +525,150 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15.6" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" defaultColWidth="11" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.796875" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="26.296875" customWidth="1"/>
-    <col min="4" max="4" width="32.19921875" customWidth="1"/>
-    <col min="5" max="5" width="23.796875" customWidth="1"/>
-    <col min="6" max="6" width="21.296875" customWidth="1"/>
+    <col min="1" max="1" width="31.6640625" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="4" width="26.1640625" customWidth="1"/>
+    <col min="5" max="5" width="18.1640625" customWidth="1"/>
+    <col min="6" max="6" width="31" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" ht="16.2" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" ht="33" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.2"/>
+    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="15.6" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" defaultColWidth="8.59765625" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:G113"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.19921875" customWidth="1"/>
+    <col min="1" max="1" width="38.6640625" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="12.296875" customWidth="1"/>
-    <col min="4" max="4" width="13.8984375" customWidth="1"/>
-    <col min="5" max="5" width="26.8984375" customWidth="1"/>
-    <col min="6" max="6" width="31" customWidth="1"/>
-    <col min="7" max="7" width="21.296875" customWidth="1"/>
+    <col min="3" max="3" width="38.6640625" customWidth="1"/>
+    <col min="4" max="4" width="37.1640625" customWidth="1"/>
+    <col min="5" max="5" width="36.6640625" customWidth="1"/>
+    <col min="6" max="6" width="19.1640625" customWidth="1"/>
+    <col min="7" max="7" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" ht="16.2" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" ht="33" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>7</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>21</v>
@@ -646,33 +686,346 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="E9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="E11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="E12" s="9"/>
+    </row>
+    <row r="13" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="E13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="E14" s="9"/>
+    </row>
+    <row r="15" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="E15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="E16" s="9"/>
+    </row>
+    <row r="17" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E17" s="9"/>
+    </row>
+    <row r="18" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E18" s="9"/>
+    </row>
+    <row r="19" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E19" s="9"/>
+    </row>
+    <row r="20" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E20" s="9"/>
+    </row>
+    <row r="21" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E21" s="9"/>
+    </row>
+    <row r="22" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E22" s="9"/>
+    </row>
+    <row r="23" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E23" s="9"/>
+    </row>
+    <row r="24" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E24" s="9"/>
+    </row>
+    <row r="25" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E25" s="9"/>
+    </row>
+    <row r="26" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E26" s="9"/>
+    </row>
+    <row r="27" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E27" s="9"/>
+    </row>
+    <row r="28" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E28" s="9"/>
+    </row>
+    <row r="29" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E29" s="9"/>
+    </row>
+    <row r="30" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E30" s="9"/>
+    </row>
+    <row r="31" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E31" s="9"/>
+    </row>
+    <row r="32" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E32" s="9"/>
+    </row>
+    <row r="33" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E33" s="9"/>
+    </row>
+    <row r="34" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E34" s="9"/>
+    </row>
+    <row r="35" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E35" s="9"/>
+    </row>
+    <row r="36" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E36" s="9"/>
+    </row>
+    <row r="37" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E37" s="9"/>
+    </row>
+    <row r="38" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E38" s="9"/>
+    </row>
+    <row r="39" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E39" s="9"/>
+    </row>
+    <row r="40" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E40" s="9"/>
+    </row>
+    <row r="41" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E41" s="9"/>
+    </row>
+    <row r="42" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E42" s="9"/>
+    </row>
+    <row r="43" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E43" s="9"/>
+    </row>
+    <row r="44" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E44" s="9"/>
+    </row>
+    <row r="45" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E45" s="9"/>
+    </row>
+    <row r="46" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E46" s="9"/>
+    </row>
+    <row r="47" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E47" s="9"/>
+    </row>
+    <row r="48" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E48" s="9"/>
+    </row>
+    <row r="49" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E49" s="9"/>
+    </row>
+    <row r="50" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E50" s="9"/>
+    </row>
+    <row r="51" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E51" s="9"/>
+    </row>
+    <row r="52" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E52" s="9"/>
+    </row>
+    <row r="53" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E53" s="9"/>
+    </row>
+    <row r="54" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E54" s="9"/>
+    </row>
+    <row r="55" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E55" s="9"/>
+    </row>
+    <row r="56" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E56" s="9"/>
+    </row>
+    <row r="57" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E57" s="9"/>
+    </row>
+    <row r="58" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E58" s="9"/>
+    </row>
+    <row r="59" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E59" s="9"/>
+    </row>
+    <row r="60" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E60" s="9"/>
+    </row>
+    <row r="61" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E61" s="9"/>
+    </row>
+    <row r="62" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E62" s="9"/>
+    </row>
+    <row r="63" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E63" s="9"/>
+    </row>
+    <row r="64" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E64" s="9"/>
+    </row>
+    <row r="65" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E65" s="9"/>
+    </row>
+    <row r="66" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E66" s="9"/>
+    </row>
+    <row r="67" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E67" s="9"/>
+    </row>
+    <row r="68" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E68" s="9"/>
+    </row>
+    <row r="69" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E69" s="9"/>
+    </row>
+    <row r="70" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E70" s="9"/>
+    </row>
+    <row r="71" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E71" s="9"/>
+    </row>
+    <row r="72" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E72" s="9"/>
+    </row>
+    <row r="73" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E73" s="9"/>
+    </row>
+    <row r="74" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E74" s="9"/>
+    </row>
+    <row r="75" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E75" s="9"/>
+    </row>
+    <row r="76" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E76" s="9"/>
+    </row>
+    <row r="77" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E77" s="9"/>
+    </row>
+    <row r="78" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E78" s="9"/>
+    </row>
+    <row r="79" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E79" s="9"/>
+    </row>
+    <row r="80" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E80" s="9"/>
+    </row>
+    <row r="81" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E81" s="9"/>
+    </row>
+    <row r="82" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E82" s="9"/>
+    </row>
+    <row r="83" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E83" s="9"/>
+    </row>
+    <row r="84" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E84" s="9"/>
+    </row>
+    <row r="85" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E85" s="9"/>
+    </row>
+    <row r="86" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E86" s="9"/>
+    </row>
+    <row r="87" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E87" s="9"/>
+    </row>
+    <row r="88" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E88" s="9"/>
+    </row>
+    <row r="89" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E89" s="9"/>
+    </row>
+    <row r="90" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E90" s="9"/>
+    </row>
+    <row r="91" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E91" s="9"/>
+    </row>
+    <row r="92" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E92" s="9"/>
+    </row>
+    <row r="93" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E93" s="9"/>
+    </row>
+    <row r="94" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E94" s="9"/>
+    </row>
+    <row r="95" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E95" s="9"/>
+    </row>
+    <row r="96" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E96" s="9"/>
+    </row>
+    <row r="97" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E97" s="9"/>
+    </row>
+    <row r="98" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E98" s="9"/>
+    </row>
+    <row r="99" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E99" s="9"/>
+    </row>
+    <row r="100" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E100" s="9"/>
+    </row>
+    <row r="101" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E101" s="9"/>
+    </row>
+    <row r="102" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E102" s="9"/>
+    </row>
+    <row r="103" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E103" s="9"/>
+    </row>
+    <row r="104" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E104" s="9"/>
+    </row>
+    <row r="105" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E105" s="9"/>
+    </row>
+    <row r="106" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E106" s="9"/>
+    </row>
+    <row r="107" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E107" s="9"/>
+    </row>
+    <row r="108" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E108" s="9"/>
+    </row>
+    <row r="109" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E109" s="9"/>
+    </row>
+    <row r="110" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E110" s="9"/>
+    </row>
+    <row r="111" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E111" s="9"/>
+    </row>
+    <row r="112" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E112" s="9"/>
+    </row>
+    <row r="113" spans="5:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="E113" s="9"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>